<commit_message>
Enhance vendor retrieval and access control for clients and internal users
</commit_message>
<xml_diff>
--- a/uploads/Employee_Record_Template.xlsx
+++ b/uploads/Employee_Record_Template.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hp\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hp\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5031DDA-0D53-4A8A-85CA-61248DBB1814}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21AFEEC6-4E88-439B-86D9-BB93B2E15227}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -103,13 +103,13 @@
     <t>rishi</t>
   </si>
   <si>
-    <t>Basic</t>
+    <t xml:space="preserve">Basic </t>
+  </si>
+  <si>
+    <t>Any Other Allowance</t>
   </si>
   <si>
     <t>Gross</t>
-  </si>
-  <si>
-    <t>Any Other Allowance</t>
   </si>
 </sst>
 </file>
@@ -567,7 +567,7 @@
         <v>6</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>7</v>
@@ -579,7 +579,7 @@
         <v>9</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="N1" s="1" t="s">
         <v>10</v>

</xml_diff>

<commit_message>
Add initial backend structure and models for user, document, and vendor
</commit_message>
<xml_diff>
--- a/uploads/Employee_Record_Template.xlsx
+++ b/uploads/Employee_Record_Template.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hp\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hp\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21AFEEC6-4E88-439B-86D9-BB93B2E15227}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5031DDA-0D53-4A8A-85CA-61248DBB1814}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -103,13 +103,13 @@
     <t>rishi</t>
   </si>
   <si>
-    <t xml:space="preserve">Basic </t>
+    <t>Basic</t>
+  </si>
+  <si>
+    <t>Gross</t>
   </si>
   <si>
     <t>Any Other Allowance</t>
-  </si>
-  <si>
-    <t>Gross</t>
   </si>
 </sst>
 </file>
@@ -567,7 +567,7 @@
         <v>6</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>7</v>
@@ -579,7 +579,7 @@
         <v>9</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="N1" s="1" t="s">
         <v>10</v>

</xml_diff>